<commit_message>
updated some benchmark related files
</commit_message>
<xml_diff>
--- a/benchmarks_tests/FINAL_Benchmarks_for_paper/PyFock_scaling_behavior_GPU.xlsx
+++ b/benchmarks_tests/FINAL_Benchmarks_for_paper/PyFock_scaling_behavior_GPU.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/manas/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/manas/Documents/PyFock/benchmarks_tests/FINAL_Benchmarks_for_paper/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72F829CD-50EA-D64D-8EEA-AB7F054EB4A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC957A0E-DA30-A844-8568-79120B984C1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1360" yWindow="760" windowWidth="28040" windowHeight="16960" xr2:uid="{580CF0B2-FD39-1547-AD8E-82680C382266}"/>
   </bookViews>
@@ -3259,29 +3259,23 @@
       <c r="B8">
         <v>125</v>
       </c>
-      <c r="C8" s="1">
-        <v>2.9560983460396502</v>
-      </c>
-      <c r="D8" s="1">
-        <v>0.42427957803010902</v>
-      </c>
-      <c r="E8" s="1">
-        <v>0.86814015824347701</v>
-      </c>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
       <c r="F8" s="1">
         <v>10</v>
       </c>
       <c r="G8">
         <f t="shared" ref="G8:G15" si="0">C8/F8</f>
-        <v>0.295609834603965</v>
+        <v>0</v>
       </c>
       <c r="H8">
         <f t="shared" ref="H8:H15" si="1">D8/F8</f>
-        <v>4.2427957803010903E-2</v>
+        <v>0</v>
       </c>
       <c r="I8">
         <f t="shared" ref="I8:I15" si="2">E8/F8</f>
-        <v>8.6814015824347696E-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
@@ -3324,28 +3318,28 @@
         <v>500</v>
       </c>
       <c r="C10" s="1">
-        <v>6.0103211449459097</v>
+        <v>5.7691683680750403</v>
       </c>
       <c r="D10" s="1">
-        <v>2.4581313524395201</v>
+        <v>2.1158297739457299</v>
       </c>
       <c r="E10" s="1">
-        <v>1.7156712030991901</v>
+        <v>2.0066158876288598</v>
       </c>
       <c r="F10" s="1">
         <v>13</v>
       </c>
       <c r="G10">
         <f t="shared" si="0"/>
-        <v>0.46233239576506996</v>
+        <v>0.44378218215961851</v>
       </c>
       <c r="H10">
         <f t="shared" si="1"/>
-        <v>0.1890870271107323</v>
+        <v>0.16275613645736384</v>
       </c>
       <c r="I10">
         <f t="shared" si="2"/>
-        <v>0.13197470793070692</v>
+        <v>0.15435506827914305</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
@@ -3356,28 +3350,28 @@
         <v>800</v>
       </c>
       <c r="C11" s="1">
-        <v>13.9464681548997</v>
+        <v>12.2090913550928</v>
       </c>
       <c r="D11" s="1">
-        <v>6.0748179610818598</v>
+        <v>5.2523773421998996</v>
       </c>
       <c r="E11" s="1">
-        <v>4.0294136004522398</v>
+        <v>3.9277749070897698</v>
       </c>
       <c r="F11" s="1">
         <v>15</v>
       </c>
       <c r="G11">
         <f t="shared" si="0"/>
-        <v>0.92976454365997996</v>
+        <v>0.81393942367285332</v>
       </c>
       <c r="H11">
         <f t="shared" si="1"/>
-        <v>0.404987864072124</v>
+        <v>0.35015848947999328</v>
       </c>
       <c r="I11">
         <f t="shared" si="2"/>
-        <v>0.26862757336348264</v>
+        <v>0.26185166047265135</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
@@ -3388,28 +3382,28 @@
         <v>1175</v>
       </c>
       <c r="C12" s="1">
-        <v>27.236856956034899</v>
+        <v>23.0492668540682</v>
       </c>
       <c r="D12" s="1">
-        <v>13.445535489358001</v>
+        <v>11.764931902987801</v>
       </c>
       <c r="E12" s="1">
-        <v>7.2065506465732998</v>
+        <v>6.2060886947438103</v>
       </c>
       <c r="F12" s="1">
         <v>15</v>
       </c>
       <c r="G12">
         <f t="shared" si="0"/>
-        <v>1.8157904637356599</v>
+        <v>1.5366177902712133</v>
       </c>
       <c r="H12">
         <f t="shared" si="1"/>
-        <v>0.89636903262386669</v>
+        <v>0.78432879353252005</v>
       </c>
       <c r="I12">
         <f t="shared" si="2"/>
-        <v>0.48043670977155334</v>
+        <v>0.41373924631625403</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
@@ -3420,28 +3414,28 @@
         <v>1900</v>
       </c>
       <c r="C13" s="1">
-        <v>69.871257518418105</v>
+        <v>55.972384363878497</v>
       </c>
       <c r="D13" s="1">
-        <v>36.925900157541001</v>
+        <v>31.8730793460272</v>
       </c>
       <c r="E13" s="1">
-        <v>16.8591308072209</v>
+        <v>13.263924242928599</v>
       </c>
       <c r="F13" s="1">
         <v>17</v>
       </c>
       <c r="G13">
         <f t="shared" si="0"/>
-        <v>4.1100739716716532</v>
+        <v>3.2924931978752059</v>
       </c>
       <c r="H13">
         <f t="shared" si="1"/>
-        <v>2.172111773973</v>
+        <v>1.8748870203545411</v>
       </c>
       <c r="I13">
         <f t="shared" si="2"/>
-        <v>0.99171357689534712</v>
+        <v>0.78023083781932934</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
@@ -3452,28 +3446,28 @@
         <v>2500</v>
       </c>
       <c r="C14" s="1">
-        <v>114.97582897730101</v>
+        <v>88.581307347165406</v>
       </c>
       <c r="D14" s="1">
-        <v>67.9061539517715</v>
+        <v>57.356785830110297</v>
       </c>
       <c r="E14" s="1">
-        <v>20.950647555291599</v>
+        <v>16.1813672701828</v>
       </c>
       <c r="F14" s="1">
         <v>15</v>
       </c>
       <c r="G14">
         <f t="shared" si="0"/>
-        <v>7.6650552651534003</v>
+        <v>5.9054204898110267</v>
       </c>
       <c r="H14">
         <f t="shared" si="1"/>
-        <v>4.5270769301181</v>
+        <v>3.823785722007353</v>
       </c>
       <c r="I14">
         <f t="shared" si="2"/>
-        <v>1.39670983701944</v>
+        <v>1.0787578180121866</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
@@ -3484,28 +3478,28 @@
         <v>3475</v>
       </c>
       <c r="C15" s="1">
-        <v>231.74738594610201</v>
+        <v>171.51697664405199</v>
       </c>
       <c r="D15" s="1">
-        <v>136.71365584619301</v>
+        <v>114.241373233031</v>
       </c>
       <c r="E15" s="1">
-        <v>35.890776604413901</v>
+        <v>26.2381101583596</v>
       </c>
       <c r="F15" s="1">
         <v>16</v>
       </c>
       <c r="G15">
         <f t="shared" si="0"/>
-        <v>14.484211621631376</v>
+        <v>10.71981104025325</v>
       </c>
       <c r="H15">
         <f t="shared" si="1"/>
-        <v>8.5446034903870629</v>
+        <v>7.1400858270644374</v>
       </c>
       <c r="I15">
         <f t="shared" si="2"/>
-        <v>2.2431735377758688</v>
+        <v>1.639881884897475</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
@@ -3752,6 +3746,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>